<commit_message>
include no CO2 result tables
</commit_message>
<xml_diff>
--- a/Plotting/Latex/filtered_data_sensitivity.xlsx
+++ b/Plotting/Latex/filtered_data_sensitivity.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R50"/>
+  <dimension ref="A1:X50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,19 +472,25 @@
       <c r="G1" s="1" t="n"/>
       <c r="H1" s="1" t="n"/>
       <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Brownfield (Scope 1, 2, and 3)</t>
-        </is>
-      </c>
+      <c r="J1" s="1" t="n"/>
       <c r="K1" s="1" t="n"/>
       <c r="L1" s="1" t="n"/>
-      <c r="M1" s="1" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Brownfield (Scope 1, 2, and 3)</t>
+        </is>
+      </c>
       <c r="N1" s="1" t="n"/>
       <c r="O1" s="1" t="n"/>
       <c r="P1" s="1" t="n"/>
       <c r="Q1" s="1" t="n"/>
       <c r="R1" s="1" t="n"/>
+      <c r="S1" s="1" t="n"/>
+      <c r="T1" s="1" t="n"/>
+      <c r="U1" s="1" t="n"/>
+      <c r="V1" s="1" t="n"/>
+      <c r="W1" s="1" t="n"/>
+      <c r="X1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -508,25 +514,39 @@
       <c r="I2" s="1" t="n"/>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t>Direct Emissions from MPW Gasification</t>
+          <t>No \ce{CO2} electrolyzers</t>
         </is>
       </c>
       <c r="K2" s="1" t="n"/>
       <c r="L2" s="1" t="n"/>
       <c r="M2" s="1" t="inlineStr">
         <is>
-          <t>Optimistic Bio-Feedstock Prices</t>
+          <t>Direct Emissions from MPW Gasification</t>
         </is>
       </c>
       <c r="N2" s="1" t="n"/>
       <c r="O2" s="1" t="n"/>
       <c r="P2" s="1" t="inlineStr">
         <is>
-          <t>Tighter Short-Term Emission Limit</t>
+          <t>Optimistic Bio-Feedstock Prices</t>
         </is>
       </c>
       <c r="Q2" s="1" t="n"/>
       <c r="R2" s="1" t="n"/>
+      <c r="S2" s="1" t="inlineStr">
+        <is>
+          <t>No \ce{CO2} electrolyzers</t>
+        </is>
+      </c>
+      <c r="T2" s="1" t="n"/>
+      <c r="U2" s="1" t="n"/>
+      <c r="V2" s="1" t="inlineStr">
+        <is>
+          <t>Tighter Short-Term Emission Limit</t>
+        </is>
+      </c>
+      <c r="W2" s="1" t="n"/>
+      <c r="X2" s="1" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -617,6 +637,36 @@
           <t>Long-term</t>
         </is>
       </c>
+      <c r="S3" s="1" t="inlineStr">
+        <is>
+          <t>Short-term</t>
+        </is>
+      </c>
+      <c r="T3" s="1" t="inlineStr">
+        <is>
+          <t>Mid-term</t>
+        </is>
+      </c>
+      <c r="U3" s="1" t="inlineStr">
+        <is>
+          <t>Long-term</t>
+        </is>
+      </c>
+      <c r="V3" s="1" t="inlineStr">
+        <is>
+          <t>Short-term</t>
+        </is>
+      </c>
+      <c r="W3" s="1" t="inlineStr">
+        <is>
+          <t>Mid-term</t>
+        </is>
+      </c>
+      <c r="X3" s="1" t="inlineStr">
+        <is>
+          <t>Long-term</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -650,10 +700,8 @@
       <c r="I5" t="n">
         <v>0</v>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="J5" t="n">
+        <v>0</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -691,6 +739,36 @@
         </is>
       </c>
       <c r="R5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -728,10 +806,8 @@
       <c r="I6" t="n">
         <v>0</v>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="J6" t="n">
+        <v>0</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -769,6 +845,36 @@
         </is>
       </c>
       <c r="R6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -818,8 +924,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J7" t="n">
-        <v>0</v>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -853,6 +961,32 @@
         </is>
       </c>
       <c r="R7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -902,8 +1036,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J8" t="n">
-        <v>0</v>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -937,6 +1073,32 @@
         </is>
       </c>
       <c r="R8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1001,6 +1163,24 @@
       <c r="R9" t="n">
         <v>0</v>
       </c>
+      <c r="S9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -1034,10 +1214,8 @@
       <c r="I10" t="n">
         <v>0</v>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="J10" t="n">
+        <v>0</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1075,6 +1253,36 @@
         </is>
       </c>
       <c r="R10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1112,10 +1320,8 @@
       <c r="I11" t="n">
         <v>0</v>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="J11" t="n">
+        <v>0</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1153,6 +1359,36 @@
         </is>
       </c>
       <c r="R11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1202,8 +1438,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J12" t="n">
-        <v>0</v>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1237,6 +1475,32 @@
         </is>
       </c>
       <c r="R12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V12" t="n">
+        <v>0</v>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1286,8 +1550,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J13" t="n">
-        <v>0</v>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1321,6 +1587,32 @@
         </is>
       </c>
       <c r="R13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S13" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V13" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1359,7 +1651,7 @@
         <v>731</v>
       </c>
       <c r="J14" t="n">
-        <v>744</v>
+        <v>696</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -1377,12 +1669,30 @@
         <v>0</v>
       </c>
       <c r="P14" t="n">
+        <v>744</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" t="n">
+        <v>751</v>
+      </c>
+      <c r="T14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" t="n">
         <v>739</v>
       </c>
-      <c r="Q14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" t="n">
+      <c r="W14" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1435,11 +1745,15 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K15" t="n">
-        <v>744</v>
-      </c>
-      <c r="L15" t="n">
-        <v>744</v>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -1458,9 +1772,31 @@
         </is>
       </c>
       <c r="Q15" t="n">
+        <v>744</v>
+      </c>
+      <c r="R15" t="n">
+        <v>744</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T15" t="n">
+        <v>751</v>
+      </c>
+      <c r="U15" t="n">
+        <v>751</v>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W15" t="n">
         <v>739</v>
       </c>
-      <c r="R15" t="n">
+      <c r="X15" t="n">
         <v>739</v>
       </c>
     </row>
@@ -1497,30 +1833,48 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>236</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>1330</v>
       </c>
       <c r="L16" t="n">
+        <v>2160</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
         <v>5</v>
       </c>
-      <c r="M16" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" t="n">
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="n">
         <v>20</v>
       </c>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="n">
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" t="n">
+        <v>147</v>
+      </c>
+      <c r="T16" t="n">
+        <v>622</v>
+      </c>
+      <c r="U16" t="n">
+        <v>465</v>
+      </c>
+      <c r="V16" t="n">
         <v>192</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="W16" t="n">
         <v>75</v>
       </c>
-      <c r="R16" t="n">
+      <c r="X16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1593,18 +1947,44 @@
           <t>-</t>
         </is>
       </c>
-      <c r="O17" t="n">
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R17" t="n">
         <v>20</v>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q17" t="n">
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T17" t="n">
+        <v>147</v>
+      </c>
+      <c r="U17" t="n">
+        <v>770</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W17" t="n">
         <v>192</v>
       </c>
-      <c r="R17" t="n">
+      <c r="X17" t="n">
         <v>268</v>
       </c>
     </row>
@@ -1641,13 +2021,13 @@
         <v>803</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>844</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>850</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>803</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
@@ -1665,6 +2045,24 @@
         <v>0</v>
       </c>
       <c r="R18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" t="n">
+        <v>0</v>
+      </c>
+      <c r="W18" t="n">
+        <v>0</v>
+      </c>
+      <c r="X18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1712,14 +2110,20 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J19" t="n">
-        <v>813</v>
-      </c>
-      <c r="K19" t="n">
-        <v>813</v>
-      </c>
-      <c r="L19" t="n">
-        <v>813</v>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M19" t="n">
         <v>813</v>
@@ -1737,6 +2141,24 @@
         <v>813</v>
       </c>
       <c r="R19" t="n">
+        <v>813</v>
+      </c>
+      <c r="S19" t="n">
+        <v>813</v>
+      </c>
+      <c r="T19" t="n">
+        <v>813</v>
+      </c>
+      <c r="U19" t="n">
+        <v>813</v>
+      </c>
+      <c r="V19" t="n">
+        <v>813</v>
+      </c>
+      <c r="W19" t="n">
+        <v>813</v>
+      </c>
+      <c r="X19" t="n">
         <v>813</v>
       </c>
     </row>
@@ -1799,6 +2221,24 @@
       <c r="R20" t="n">
         <v>0</v>
       </c>
+      <c r="S20" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" t="n">
+        <v>56</v>
+      </c>
+      <c r="V20" t="n">
+        <v>0</v>
+      </c>
+      <c r="W20" t="n">
+        <v>0</v>
+      </c>
+      <c r="X20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -1845,7 +2285,7 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -1867,6 +2307,28 @@
         <v>0</v>
       </c>
       <c r="R21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W21" t="n">
+        <v>0</v>
+      </c>
+      <c r="X21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1903,30 +2365,48 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>253</v>
+        <v>496</v>
       </c>
       <c r="K22" t="n">
-        <v>27</v>
+        <v>560</v>
       </c>
       <c r="L22" t="n">
-        <v>0</v>
+        <v>664</v>
       </c>
       <c r="M22" t="n">
         <v>253</v>
       </c>
       <c r="N22" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="O22" t="n">
         <v>0</v>
       </c>
       <c r="P22" t="n">
+        <v>253</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" t="n">
         <v>496</v>
       </c>
-      <c r="Q22" t="n">
-        <v>0</v>
-      </c>
-      <c r="R22" t="n">
+      <c r="T22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" t="n">
+        <v>46</v>
+      </c>
+      <c r="V22" t="n">
+        <v>496</v>
+      </c>
+      <c r="W22" t="n">
+        <v>0</v>
+      </c>
+      <c r="X22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1979,11 +2459,15 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K23" t="n">
-        <v>253</v>
-      </c>
-      <c r="L23" t="n">
-        <v>280</v>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -1994,17 +2478,39 @@
         <v>253</v>
       </c>
       <c r="O23" t="n">
+        <v>280</v>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q23" t="n">
         <v>253</v>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q23" t="n">
+      <c r="R23" t="n">
+        <v>253</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T23" t="n">
         <v>496</v>
       </c>
-      <c r="R23" t="n">
+      <c r="U23" t="n">
+        <v>496</v>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W23" t="n">
+        <v>496</v>
+      </c>
+      <c r="X23" t="n">
         <v>496</v>
       </c>
     </row>
@@ -2067,6 +2573,24 @@
       <c r="R24" t="n">
         <v>0</v>
       </c>
+      <c r="S24" t="n">
+        <v>0</v>
+      </c>
+      <c r="T24" t="n">
+        <v>0</v>
+      </c>
+      <c r="U24" t="n">
+        <v>0</v>
+      </c>
+      <c r="V24" t="n">
+        <v>0</v>
+      </c>
+      <c r="W24" t="n">
+        <v>0</v>
+      </c>
+      <c r="X24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -2101,10 +2625,10 @@
         <v>157</v>
       </c>
       <c r="J25" t="n">
-        <v>157</v>
+        <v>64</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
@@ -2119,12 +2643,30 @@
         <v>0</v>
       </c>
       <c r="P25" t="n">
+        <v>157</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" t="n">
         <v>64</v>
       </c>
-      <c r="Q25" t="n">
-        <v>0</v>
-      </c>
-      <c r="R25" t="n">
+      <c r="T25" t="n">
+        <v>0</v>
+      </c>
+      <c r="U25" t="n">
+        <v>0</v>
+      </c>
+      <c r="V25" t="n">
+        <v>64</v>
+      </c>
+      <c r="W25" t="n">
+        <v>0</v>
+      </c>
+      <c r="X25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2177,11 +2719,15 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K26" t="n">
-        <v>157</v>
-      </c>
-      <c r="L26" t="n">
-        <v>157</v>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
@@ -2200,9 +2746,31 @@
         </is>
       </c>
       <c r="Q26" t="n">
+        <v>157</v>
+      </c>
+      <c r="R26" t="n">
+        <v>157</v>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T26" t="n">
         <v>64</v>
       </c>
-      <c r="R26" t="n">
+      <c r="U26" t="n">
+        <v>64</v>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W26" t="n">
+        <v>64</v>
+      </c>
+      <c r="X26" t="n">
         <v>64</v>
       </c>
     </row>
@@ -2239,30 +2807,48 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>172</v>
+        <v>338</v>
       </c>
       <c r="K27" t="n">
-        <v>18</v>
+        <v>381</v>
       </c>
       <c r="L27" t="n">
-        <v>0</v>
+        <v>395</v>
       </c>
       <c r="M27" t="n">
         <v>172</v>
       </c>
       <c r="N27" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="O27" t="n">
         <v>0</v>
       </c>
       <c r="P27" t="n">
+        <v>172</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" t="n">
         <v>338</v>
       </c>
-      <c r="Q27" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" t="n">
+      <c r="T27" t="n">
+        <v>0</v>
+      </c>
+      <c r="U27" t="n">
+        <v>0</v>
+      </c>
+      <c r="V27" t="n">
+        <v>338</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0</v>
+      </c>
+      <c r="X27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2302,27 +2888,45 @@
         <v>0</v>
       </c>
       <c r="K28" t="n">
+        <v>10</v>
+      </c>
+      <c r="L28" t="n">
+        <v>31</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" t="n">
         <v>87</v>
       </c>
-      <c r="L28" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" t="n">
-        <v>0</v>
-      </c>
       <c r="O28" t="n">
         <v>0</v>
       </c>
       <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" t="n">
+        <v>0</v>
+      </c>
+      <c r="U28" t="n">
+        <v>0</v>
+      </c>
+      <c r="V28" t="n">
         <v>3</v>
       </c>
-      <c r="Q28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" t="n">
+      <c r="W28" t="n">
+        <v>0</v>
+      </c>
+      <c r="X28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2375,11 +2979,15 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K29" t="n">
-        <v>172</v>
-      </c>
-      <c r="L29" t="n">
-        <v>190</v>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -2390,17 +2998,39 @@
         <v>172</v>
       </c>
       <c r="O29" t="n">
+        <v>190</v>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q29" t="n">
         <v>172</v>
       </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q29" t="n">
+      <c r="R29" t="n">
+        <v>172</v>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T29" t="n">
         <v>338</v>
       </c>
-      <c r="R29" t="n">
+      <c r="U29" t="n">
+        <v>338</v>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W29" t="n">
+        <v>338</v>
+      </c>
+      <c r="X29" t="n">
         <v>338</v>
       </c>
     </row>
@@ -2453,11 +3083,15 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K30" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" t="n">
-        <v>0</v>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
@@ -2476,9 +3110,31 @@
         </is>
       </c>
       <c r="Q30" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T30" t="n">
+        <v>8</v>
+      </c>
+      <c r="U30" t="n">
+        <v>22</v>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W30" t="n">
         <v>28</v>
       </c>
-      <c r="R30" t="n">
+      <c r="X30" t="n">
         <v>53</v>
       </c>
     </row>
@@ -2523,32 +3179,62 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K31" t="n">
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
         <v>129</v>
       </c>
-      <c r="L31" t="n">
+      <c r="O31" t="n">
         <v>32</v>
       </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N31" t="n">
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q31" t="n">
         <v>103</v>
       </c>
-      <c r="O31" t="n">
+      <c r="R31" t="n">
         <v>38</v>
       </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q31" t="n">
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W31" t="n">
         <v>111</v>
       </c>
-      <c r="R31" t="n">
+      <c r="X31" t="n">
         <v>39</v>
       </c>
     </row>
@@ -2606,33 +3292,63 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L32" t="n">
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O32" t="n">
         <v>129</v>
       </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O32" t="n">
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R32" t="n">
         <v>103</v>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R32" t="n">
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X32" t="n">
         <v>111</v>
       </c>
     </row>
@@ -2669,13 +3385,13 @@
         <v>27</v>
       </c>
       <c r="J33" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K33" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="L33" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="M33" t="n">
         <v>28</v>
@@ -2693,6 +3409,24 @@
         <v>0</v>
       </c>
       <c r="R33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" t="n">
+        <v>28</v>
+      </c>
+      <c r="T33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V33" t="n">
+        <v>28</v>
+      </c>
+      <c r="W33" t="n">
+        <v>0</v>
+      </c>
+      <c r="X33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2745,11 +3479,15 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K34" t="n">
-        <v>28</v>
-      </c>
-      <c r="L34" t="n">
-        <v>28</v>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
@@ -2771,6 +3509,28 @@
         <v>28</v>
       </c>
       <c r="R34" t="n">
+        <v>28</v>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T34" t="n">
+        <v>28</v>
+      </c>
+      <c r="U34" t="n">
+        <v>28</v>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W34" t="n">
+        <v>28</v>
+      </c>
+      <c r="X34" t="n">
         <v>28</v>
       </c>
     </row>
@@ -2807,30 +3567,48 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
+        <v>128</v>
+      </c>
+      <c r="K35" t="n">
+        <v>63</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" t="n">
         <v>355</v>
       </c>
-      <c r="K35" t="n">
+      <c r="N35" t="n">
         <v>11</v>
       </c>
-      <c r="L35" t="n">
-        <v>0</v>
-      </c>
-      <c r="M35" t="n">
+      <c r="O35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" t="n">
         <v>367</v>
       </c>
-      <c r="N35" t="n">
-        <v>0</v>
-      </c>
-      <c r="O35" t="n">
-        <v>0</v>
-      </c>
-      <c r="P35" t="n">
+      <c r="Q35" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" t="n">
+        <v>124</v>
+      </c>
+      <c r="T35" t="n">
+        <v>5</v>
+      </c>
+      <c r="U35" t="n">
+        <v>0</v>
+      </c>
+      <c r="V35" t="n">
         <v>122</v>
       </c>
-      <c r="Q35" t="n">
-        <v>0</v>
-      </c>
-      <c r="R35" t="n">
+      <c r="W35" t="n">
+        <v>0</v>
+      </c>
+      <c r="X35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2883,19 +3661,23 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K36" t="n">
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N36" t="n">
         <v>355</v>
-      </c>
-      <c r="L36" t="n">
-        <v>367</v>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N36" t="n">
-        <v>367</v>
       </c>
       <c r="O36" t="n">
         <v>367</v>
@@ -2906,9 +3688,31 @@
         </is>
       </c>
       <c r="Q36" t="n">
+        <v>367</v>
+      </c>
+      <c r="R36" t="n">
+        <v>367</v>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T36" t="n">
+        <v>124</v>
+      </c>
+      <c r="U36" t="n">
+        <v>129</v>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W36" t="n">
         <v>122</v>
       </c>
-      <c r="R36" t="n">
+      <c r="X36" t="n">
         <v>122</v>
       </c>
     </row>
@@ -2945,13 +3749,13 @@
         <v>294</v>
       </c>
       <c r="J37" t="n">
-        <v>293</v>
+        <v>65</v>
       </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="L37" t="n">
-        <v>0</v>
+        <v>124</v>
       </c>
       <c r="M37" t="n">
         <v>293</v>
@@ -2963,12 +3767,30 @@
         <v>0</v>
       </c>
       <c r="P37" t="n">
+        <v>293</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" t="n">
+        <v>64</v>
+      </c>
+      <c r="T37" t="n">
+        <v>91</v>
+      </c>
+      <c r="U37" t="n">
+        <v>56</v>
+      </c>
+      <c r="V37" t="n">
         <v>97</v>
       </c>
-      <c r="Q37" t="n">
-        <v>0</v>
-      </c>
-      <c r="R37" t="n">
+      <c r="W37" t="n">
+        <v>0</v>
+      </c>
+      <c r="X37" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3021,11 +3843,15 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K38" t="n">
-        <v>293</v>
-      </c>
-      <c r="L38" t="n">
-        <v>293</v>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
@@ -3044,9 +3870,31 @@
         </is>
       </c>
       <c r="Q38" t="n">
+        <v>293</v>
+      </c>
+      <c r="R38" t="n">
+        <v>293</v>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T38" t="n">
+        <v>64</v>
+      </c>
+      <c r="U38" t="n">
+        <v>155</v>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W38" t="n">
         <v>97</v>
       </c>
-      <c r="R38" t="n">
+      <c r="X38" t="n">
         <v>97</v>
       </c>
     </row>
@@ -3083,30 +3931,48 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
+        <v>7907</v>
+      </c>
+      <c r="K39" t="n">
+        <v>11258</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" t="n">
         <v>3358</v>
       </c>
-      <c r="K39" t="n">
+      <c r="N39" t="n">
         <v>5389</v>
       </c>
-      <c r="L39" t="n">
-        <v>0</v>
-      </c>
-      <c r="M39" t="n">
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="n">
         <v>3656</v>
       </c>
-      <c r="N39" t="n">
+      <c r="Q39" t="n">
         <v>5433</v>
       </c>
-      <c r="O39" t="n">
-        <v>0</v>
-      </c>
-      <c r="P39" t="n">
+      <c r="R39" t="n">
+        <v>0</v>
+      </c>
+      <c r="S39" t="n">
+        <v>4209</v>
+      </c>
+      <c r="T39" t="n">
+        <v>4906</v>
+      </c>
+      <c r="U39" t="n">
+        <v>0</v>
+      </c>
+      <c r="V39" t="n">
         <v>4513</v>
       </c>
-      <c r="Q39" t="n">
+      <c r="W39" t="n">
         <v>4602</v>
       </c>
-      <c r="R39" t="n">
+      <c r="X39" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3159,32 +4025,58 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K40" t="n">
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N40" t="n">
         <v>3358</v>
       </c>
-      <c r="L40" t="n">
+      <c r="O40" t="n">
         <v>8747</v>
       </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N40" t="n">
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q40" t="n">
         <v>3656</v>
       </c>
-      <c r="O40" t="n">
+      <c r="R40" t="n">
         <v>9089</v>
       </c>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q40" t="n">
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T40" t="n">
+        <v>4209</v>
+      </c>
+      <c r="U40" t="n">
+        <v>9116</v>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W40" t="n">
         <v>4513</v>
       </c>
-      <c r="R40" t="n">
+      <c r="X40" t="n">
         <v>9116</v>
       </c>
     </row>
@@ -3221,7 +4113,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>1470</v>
+        <v>1219</v>
       </c>
       <c r="K41" t="n">
         <v>6414</v>
@@ -3230,7 +4122,7 @@
         <v>0</v>
       </c>
       <c r="M41" t="n">
-        <v>1432</v>
+        <v>1470</v>
       </c>
       <c r="N41" t="n">
         <v>6414</v>
@@ -3239,12 +4131,30 @@
         <v>0</v>
       </c>
       <c r="P41" t="n">
-        <v>1639</v>
+        <v>1432</v>
       </c>
       <c r="Q41" t="n">
         <v>6414</v>
       </c>
       <c r="R41" t="n">
+        <v>0</v>
+      </c>
+      <c r="S41" t="n">
+        <v>1662</v>
+      </c>
+      <c r="T41" t="n">
+        <v>6414</v>
+      </c>
+      <c r="U41" t="n">
+        <v>0</v>
+      </c>
+      <c r="V41" t="n">
+        <v>1639</v>
+      </c>
+      <c r="W41" t="n">
+        <v>6414</v>
+      </c>
+      <c r="X41" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3297,32 +4207,58 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K42" t="n">
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N42" t="n">
         <v>1470</v>
       </c>
-      <c r="L42" t="n">
+      <c r="O42" t="n">
         <v>7884</v>
       </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N42" t="n">
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q42" t="n">
         <v>1432</v>
       </c>
-      <c r="O42" t="n">
+      <c r="R42" t="n">
         <v>7846</v>
       </c>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q42" t="n">
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T42" t="n">
+        <v>1662</v>
+      </c>
+      <c r="U42" t="n">
+        <v>8076</v>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W42" t="n">
         <v>1639</v>
       </c>
-      <c r="R42" t="n">
+      <c r="X42" t="n">
         <v>8053</v>
       </c>
     </row>
@@ -3362,27 +4298,45 @@
         <v>0</v>
       </c>
       <c r="K43" t="n">
+        <v>5221</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" t="n">
         <v>1618</v>
       </c>
-      <c r="L43" t="n">
-        <v>0</v>
-      </c>
-      <c r="M43" t="n">
-        <v>0</v>
-      </c>
-      <c r="N43" t="n">
+      <c r="O43" t="n">
+        <v>0</v>
+      </c>
+      <c r="P43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q43" t="n">
         <v>117</v>
       </c>
-      <c r="O43" t="n">
+      <c r="R43" t="n">
         <v>150</v>
       </c>
-      <c r="P43" t="n">
+      <c r="S43" t="n">
+        <v>0</v>
+      </c>
+      <c r="T43" t="n">
+        <v>0</v>
+      </c>
+      <c r="U43" t="n">
+        <v>0</v>
+      </c>
+      <c r="V43" t="n">
         <v>2135</v>
       </c>
-      <c r="Q43" t="n">
+      <c r="W43" t="n">
         <v>7669</v>
       </c>
-      <c r="R43" t="n">
+      <c r="X43" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3440,31 +4394,61 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L44" t="n">
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O44" t="n">
         <v>1618</v>
       </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O44" t="n">
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R44" t="n">
         <v>117</v>
       </c>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q44" t="n">
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W44" t="n">
         <v>2135</v>
       </c>
-      <c r="R44" t="n">
+      <c r="X44" t="n">
         <v>9805</v>
       </c>
     </row>
@@ -3501,30 +4485,48 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
+        <v>128</v>
       </c>
       <c r="K45" t="n">
+        <v>32492</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" t="n">
         <v>494</v>
       </c>
-      <c r="L45" t="n">
-        <v>0</v>
-      </c>
-      <c r="M45" t="n">
-        <v>0</v>
-      </c>
-      <c r="N45" t="n">
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="n">
         <v>694</v>
       </c>
-      <c r="O45" t="n">
-        <v>0</v>
-      </c>
-      <c r="P45" t="n">
+      <c r="R45" t="n">
+        <v>0</v>
+      </c>
+      <c r="S45" t="n">
+        <v>195</v>
+      </c>
+      <c r="T45" t="n">
+        <v>3234</v>
+      </c>
+      <c r="U45" t="n">
+        <v>0</v>
+      </c>
+      <c r="V45" t="n">
         <v>270</v>
       </c>
-      <c r="Q45" t="n">
+      <c r="W45" t="n">
         <v>8471</v>
       </c>
-      <c r="R45" t="n">
+      <c r="X45" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3582,31 +4584,57 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L46" t="n">
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O46" t="n">
         <v>494</v>
       </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O46" t="n">
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R46" t="n">
         <v>694</v>
       </c>
-      <c r="P46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q46" t="n">
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T46" t="n">
+        <v>195</v>
+      </c>
+      <c r="U46" t="n">
+        <v>3429</v>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W46" t="n">
         <v>270</v>
       </c>
-      <c r="R46" t="n">
+      <c r="X46" t="n">
         <v>8741</v>
       </c>
     </row>
@@ -3646,27 +4674,45 @@
         <v>0</v>
       </c>
       <c r="K47" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" t="n">
         <v>1133</v>
       </c>
-      <c r="L47" t="n">
-        <v>0</v>
-      </c>
-      <c r="M47" t="n">
-        <v>0</v>
-      </c>
-      <c r="N47" t="n">
+      <c r="O47" t="n">
+        <v>0</v>
+      </c>
+      <c r="P47" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q47" t="n">
         <v>477</v>
       </c>
-      <c r="O47" t="n">
-        <v>0</v>
-      </c>
-      <c r="P47" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q47" t="n">
+      <c r="R47" t="n">
+        <v>0</v>
+      </c>
+      <c r="S47" t="n">
+        <v>0</v>
+      </c>
+      <c r="T47" t="n">
+        <v>0</v>
+      </c>
+      <c r="U47" t="n">
+        <v>81</v>
+      </c>
+      <c r="V47" t="n">
+        <v>0</v>
+      </c>
+      <c r="W47" t="n">
         <v>5336</v>
       </c>
-      <c r="R47" t="n">
+      <c r="X47" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3724,33 +4770,63 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L48" t="n">
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O48" t="n">
         <v>1133</v>
       </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O48" t="n">
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R48" t="n">
         <v>477</v>
       </c>
-      <c r="P48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R48" t="n">
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X48" t="n">
         <v>5336</v>
       </c>
     </row>
@@ -3790,27 +4866,45 @@
         <v>0</v>
       </c>
       <c r="K49" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" t="n">
+        <v>0</v>
+      </c>
+      <c r="N49" t="n">
         <v>6808</v>
       </c>
-      <c r="L49" t="n">
-        <v>0</v>
-      </c>
-      <c r="M49" t="n">
-        <v>0</v>
-      </c>
-      <c r="N49" t="n">
+      <c r="O49" t="n">
+        <v>0</v>
+      </c>
+      <c r="P49" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q49" t="n">
         <v>7147</v>
       </c>
-      <c r="O49" t="n">
-        <v>0</v>
-      </c>
-      <c r="P49" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q49" t="n">
+      <c r="R49" t="n">
+        <v>0</v>
+      </c>
+      <c r="S49" t="n">
+        <v>0</v>
+      </c>
+      <c r="T49" t="n">
+        <v>0</v>
+      </c>
+      <c r="U49" t="n">
+        <v>78</v>
+      </c>
+      <c r="V49" t="n">
+        <v>0</v>
+      </c>
+      <c r="W49" t="n">
         <v>498</v>
       </c>
-      <c r="R49" t="n">
+      <c r="X49" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3868,47 +4962,79 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L50" t="n">
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O50" t="n">
         <v>6808</v>
       </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O50" t="n">
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R50" t="n">
         <v>7147</v>
       </c>
-      <c r="P50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R50" t="n">
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X50" t="n">
         <v>498</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="11">
     <mergeCell ref="D2:F2"/>
     <mergeCell ref="G2:I2"/>
+    <mergeCell ref="D1:L1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="J2:L2"/>
     <mergeCell ref="P2:R2"/>
-    <mergeCell ref="J1:R1"/>
+    <mergeCell ref="M1:X1"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="M2:O2"/>
-    <mergeCell ref="D1:I1"/>
+    <mergeCell ref="S2:U2"/>
+    <mergeCell ref="V2:X2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>